<commit_message>
feat(migration): skip report banner rows in xlsx intake (QuickBooks)
A QuickBooks Online "Customer Contact List" report exported to Excel prepends
company/title/date banner rows above the column headings (Intuit tells users to
delete them). The xlsx parser treated row 1 as the header, so a raw export
mis-parsed and failed source detection.

- intake-files.ts: add findHeaderRowOffset() and skip leading banner rows in
  sheetDataToTsv() before parsing — the header + data form a run of "wide" rows,
  so sparse banner rows above are dropped. No-op when row 1 is already the
  header (every existing fixture is unaffected).
- generator: writeXlsx() gains an optional preamble; the QBO fixture now
  includes the real banner rows, exercising the skip end-to-end.
- tests: unit-cover findHeaderRowOffset (header-first + banner cases); the QBO
  detection golden now parses through the preamble.
- README: drop the "no title rows" simplification.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product-design/migration-copilot/06-fixtures/realistic-exports/quickbooks-online-customer-contact-list.xlsx
+++ b/docs/product-design/migration-copilot/06-fixtures/realistic-exports/quickbooks-online-customer-contact-list.xlsx
@@ -8,7 +8,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="163">
+  <si>
+    <t>Ledger Lane CPAs (TEST)</t>
+  </si>
+  <si>
+    <t>Customer Contact List</t>
+  </si>
+  <si>
+    <t>As of June 1, 2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
   <si>
     <t>Customer</t>
   </si>
@@ -491,656 +503,676 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>31</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H6" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H7" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" t="s">
-        <v>56</v>
-      </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H11" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="G12" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H12" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="D13" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="F13" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="G13" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E14" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="G14" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H14" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="E15" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H15" t="s">
-        <v>100</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="D16" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="F16" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="G17" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H17" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="E18" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="G18" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H18" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="F19" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H19" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="F20" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="G20" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H20" t="s">
-        <v>129</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="E21" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="G21" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E22" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="F22" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="G22" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="H22" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="D23" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="E23" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F23" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="G23" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H23" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="B24" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="C24" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="D24" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="F24" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="G24" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>135</v>
+      </c>
+      <c r="D25" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F25" t="s">
+        <v>138</v>
+      </c>
+      <c r="G25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>139</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" t="s">
+        <v>142</v>
+      </c>
+      <c r="F26" t="s">
+        <v>143</v>
+      </c>
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E27" t="s">
+        <v>148</v>
+      </c>
+      <c r="F27" t="s">
+        <v>149</v>
+      </c>
+      <c r="G27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>152</v>
+      </c>
+      <c r="D28" t="s">
         <v>153</v>
       </c>
-      <c r="B25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="E28" t="s">
         <v>154</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F28" t="s">
         <v>155</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G28" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" t="s">
         <v>156</v>
       </c>
-      <c r="F25" t="s">
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
         <v>157</v>
       </c>
-      <c r="G25" t="s">
-        <v>30</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
         <v>158</v>
+      </c>
+      <c r="D29" t="s">
+        <v>159</v>
+      </c>
+      <c r="E29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F29" t="s">
+        <v>161</v>
+      </c>
+      <c r="G29" t="s">
+        <v>34</v>
+      </c>
+      <c r="H29" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>